<commit_message>
PAUSED (task176): stage 4 round 1 asks re-sited, waiting on a fresh judge and two fresh readers
Call held 2/2 at round 1 and is frozen (450, every call figure unchanged). The child-days ask is closed in the
prompt ("counting a child once on a day") and shrunk to two statewide figures; the money device moved onto network
remittances, one remittance carrying the children of several homes, so one amount per run date and provider (both
readers' path) misses all 20 cells and one remittance is its number, run date and county office.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task176/golden/fcc_closures_2027.xlsx
+++ b/task176/golden/fcc_closures_2027.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>About 450 of the 3,081 licensed family child care homes are expected to close during 2027</t>
   </si>
@@ -55,19 +55,46 @@
     <t>Kindergarten year as in the CCAP provider payment policy, section 6 (a child turning five on or before 1 September starts that September). Homes are small and large family child care homes (Title 170, 6.40.010). Sources: licensing extract of 8 January 2027; capacity worksheets 2016 to 2026.</t>
   </si>
   <si>
-    <t>Child-days of subsidised care in family child care homes, 2026</t>
-  </si>
-  <si>
-    <t>CCAP payment lines paid in 2026, SFCC and LFCC providers, lines not voided; each child counted once a day (Monday to Friday) whatever the number of homes paid for that day.</t>
+    <t>Child-days of subsidised care in family child care homes, Allerton, 2026</t>
+  </si>
+  <si>
+    <t>CCAP payment lines, SFCC and LFCC providers, lines not voided; each child counted once on a day (Monday to Friday) whatever the number of homes paid for that day.</t>
+  </si>
+  <si>
+    <t>Half of 2026</t>
+  </si>
+  <si>
+    <t>Child-days</t>
+  </si>
+  <si>
+    <t>January to June</t>
+  </si>
+  <si>
+    <t>July to December</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>Money the subsidy paid to family child care homes, 2026 payment runs (USD)</t>
+  </si>
+  <si>
+    <t>CCAP remittances for SFCC and LFCC homes by the date of the payment run; voided remittances out, their reissues in; each remittance counted once (number, run and county office).</t>
   </si>
   <si>
     <t>Region</t>
   </si>
   <si>
-    <t>January to June</t>
-  </si>
-  <si>
-    <t>July to December</t>
+    <t>January to March</t>
+  </si>
+  <si>
+    <t>April to June</t>
+  </si>
+  <si>
+    <t>July to September</t>
+  </si>
+  <si>
+    <t>October to December</t>
   </si>
   <si>
     <t>Region 1 North</t>
@@ -86,24 +113,6 @@
   </si>
   <si>
     <t>Allerton</t>
-  </si>
-  <si>
-    <t>Money the subsidy paid to family child care homes, 2026 payment runs (USD)</t>
-  </si>
-  <si>
-    <t>CCAP remittances to SFCC and LFCC providers by the date of the payment run; voided remittances out, their reissues in; each remittance counted once.</t>
-  </si>
-  <si>
-    <t>January to March</t>
-  </si>
-  <si>
-    <t>April to June</t>
-  </si>
-  <si>
-    <t>July to September</t>
-  </si>
-  <si>
-    <t>October to December</t>
   </si>
   <si>
     <t>Prepared 14 January 2027 from the January 2027 supply folder (licensing extract of 8 January 2027).</t>
@@ -731,98 +740,53 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="3" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:2">
       <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="B5" s="3">
+        <v>125938</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="3">
-        <v>14654</v>
-      </c>
-      <c r="C5" s="3">
-        <v>16066</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+      <c r="B6" s="3">
+        <v>137949</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="3">
-        <v>53667</v>
-      </c>
-      <c r="C6" s="3">
-        <v>56957</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="3">
-        <v>17906</v>
-      </c>
-      <c r="C7" s="3">
-        <v>20791</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="3">
-        <v>21072</v>
-      </c>
-      <c r="C8" s="3">
-        <v>23008</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="3">
-        <v>18639</v>
-      </c>
-      <c r="C9" s="3">
-        <v>21127</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="9">
-        <v>125938</v>
-      </c>
-      <c r="C10" s="9">
-        <v>137949</v>
+      <c r="B7" s="9">
+        <v>263887</v>
       </c>
     </row>
   </sheetData>
@@ -841,131 +805,131 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B5" s="3">
         <v>261758</v>
       </c>
       <c r="C5" s="3">
-        <v>299144</v>
+        <v>299956</v>
       </c>
       <c r="D5" s="3">
-        <v>308776</v>
+        <v>308387</v>
       </c>
       <c r="E5" s="3">
-        <v>320951</v>
+        <v>323302</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B6" s="3">
-        <v>976233</v>
+        <v>975519</v>
       </c>
       <c r="C6" s="3">
-        <v>1060730</v>
+        <v>1059175</v>
       </c>
       <c r="D6" s="3">
-        <v>1130314</v>
+        <v>1135102</v>
       </c>
       <c r="E6" s="3">
-        <v>1140841</v>
+        <v>1137021</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B7" s="3">
-        <v>337784</v>
+        <v>337012</v>
       </c>
       <c r="C7" s="3">
-        <v>354141</v>
+        <v>353636</v>
       </c>
       <c r="D7" s="3">
-        <v>389809</v>
+        <v>391204</v>
       </c>
       <c r="E7" s="3">
-        <v>418844</v>
+        <v>421264</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B8" s="3">
-        <v>386069</v>
+        <v>387659</v>
       </c>
       <c r="C8" s="3">
-        <v>418205</v>
+        <v>418645</v>
       </c>
       <c r="D8" s="3">
-        <v>453653</v>
+        <v>450405</v>
       </c>
       <c r="E8" s="3">
-        <v>455022</v>
+        <v>455636</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B9" s="3">
-        <v>364938</v>
+        <v>365521</v>
       </c>
       <c r="C9" s="3">
-        <v>364407</v>
+        <v>362977</v>
       </c>
       <c r="D9" s="3">
-        <v>394196</v>
+        <v>400530</v>
       </c>
       <c r="E9" s="3">
-        <v>423531</v>
+        <v>418584</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="8" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B10" s="9">
-        <v>2326782</v>
+        <v>2327469</v>
       </c>
       <c r="C10" s="9">
-        <v>2496627</v>
+        <v>2494389</v>
       </c>
       <c r="D10" s="9">
-        <v>2676748</v>
+        <v>2685628</v>
       </c>
       <c r="E10" s="9">
-        <v>2759189</v>
+        <v>2755807</v>
       </c>
     </row>
   </sheetData>
@@ -983,22 +947,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task176): Ask B re-sited onto the region of the home, waiting on round 3 readers and judge
The money is filed by the region of the home that gave the care; network remittances are issued by the base
county's office for member homes in other regions, so one amount per remittance credited to the issuing office misses
every cell. The unit and the allocation are forced by the rows and the section 3 and 5 rates (SF9, SF10 asserted);
worst-route pair on readers A to D and the mirror 33.5. Call and every call figure unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task176/golden/fcc_closures_2027.xlsx
+++ b/task176/golden/fcc_closures_2027.xlsx
@@ -79,7 +79,7 @@
     <t>Money the subsidy paid to family child care homes, 2026 payment runs (USD)</t>
   </si>
   <si>
-    <t>CCAP remittances for SFCC and LFCC homes by the date of the payment run; voided remittances out, their reissues in; each remittance counted once (number, run and county office).</t>
+    <t>CCAP remittances for SFCC and LFCC homes by the date of the payment run and the region of the home that gave the care; voided remittances out, their reissues in; each remittance counted once (number, run and county office), a remittance for homes in several regions shared by its lines' pay.</t>
   </si>
   <si>
     <t>Region</t>
@@ -770,7 +770,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="3">
-        <v>125938</v>
+        <v>124773</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -778,7 +778,7 @@
         <v>17</v>
       </c>
       <c r="B6" s="3">
-        <v>137949</v>
+        <v>131302</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -786,7 +786,7 @@
         <v>18</v>
       </c>
       <c r="B7" s="9">
-        <v>263887</v>
+        <v>256075</v>
       </c>
     </row>
   </sheetData>
@@ -835,16 +835,16 @@
         <v>26</v>
       </c>
       <c r="B5" s="3">
-        <v>261758</v>
+        <v>261011</v>
       </c>
       <c r="C5" s="3">
-        <v>299956</v>
+        <v>284679</v>
       </c>
       <c r="D5" s="3">
-        <v>308387</v>
+        <v>301788</v>
       </c>
       <c r="E5" s="3">
-        <v>323302</v>
+        <v>351377</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -852,16 +852,16 @@
         <v>27</v>
       </c>
       <c r="B6" s="3">
-        <v>975519</v>
+        <v>930268</v>
       </c>
       <c r="C6" s="3">
-        <v>1059175</v>
+        <v>956164</v>
       </c>
       <c r="D6" s="3">
-        <v>1135102</v>
+        <v>950014</v>
       </c>
       <c r="E6" s="3">
-        <v>1137021</v>
+        <v>968166</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -869,16 +869,16 @@
         <v>28</v>
       </c>
       <c r="B7" s="3">
-        <v>337012</v>
+        <v>331513</v>
       </c>
       <c r="C7" s="3">
-        <v>353636</v>
+        <v>335325</v>
       </c>
       <c r="D7" s="3">
-        <v>391204</v>
+        <v>366990</v>
       </c>
       <c r="E7" s="3">
-        <v>421264</v>
+        <v>368805</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -886,16 +886,16 @@
         <v>29</v>
       </c>
       <c r="B8" s="3">
-        <v>387659</v>
+        <v>394956</v>
       </c>
       <c r="C8" s="3">
-        <v>418645</v>
+        <v>413421</v>
       </c>
       <c r="D8" s="3">
-        <v>450405</v>
+        <v>424992</v>
       </c>
       <c r="E8" s="3">
-        <v>455636</v>
+        <v>478850</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -903,16 +903,16 @@
         <v>30</v>
       </c>
       <c r="B9" s="3">
-        <v>365521</v>
+        <v>431566</v>
       </c>
       <c r="C9" s="3">
-        <v>362977</v>
+        <v>461036</v>
       </c>
       <c r="D9" s="3">
-        <v>400530</v>
+        <v>453954</v>
       </c>
       <c r="E9" s="3">
-        <v>418584</v>
+        <v>454203</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -920,16 +920,16 @@
         <v>31</v>
       </c>
       <c r="B10" s="9">
-        <v>2327469</v>
+        <v>2349314</v>
       </c>
       <c r="C10" s="9">
-        <v>2494389</v>
+        <v>2450625</v>
       </c>
       <c r="D10" s="9">
-        <v>2685628</v>
+        <v>2497738</v>
       </c>
       <c r="E10" s="9">
-        <v>2755807</v>
+        <v>2621401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task176): world retuned so the honest model family sits centred in the 450 cell, waiting on round 4 readers and judge
Round 3 found the honest models at 419 to 456 around the 425 edge. The world's kindergarten-summer excess and draw
are retuned; the golden is the family's centre, 450.4, and the 16-member family (banded and linear and no tenure,
Poisson read as probabilities and as rates, logit, fits from 2020 and 2022, annual rates) spans 437.2 to 463.6,
asserted 10 or more homes inside both edges. Child-days pinned by the date of the care; money device unchanged;
worst-route pair on all six readers 33.5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task176/golden/fcc_closures_2027.xlsx
+++ b/task176/golden/fcc_closures_2027.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
-    <t>About 450 of the 3,081 licensed family child care homes are expected to close during 2027</t>
+    <t>About 450 of the 3,051 licensed family child care homes are expected to close during 2027</t>
   </si>
   <si>
     <t>Office of Child Care, supply and planning. Input to the 2027 Home Child Care Start-Up Grant round and the supply report due 1 February 2027. Licensing record to 31 December 2026.</t>
@@ -34,10 +34,10 @@
     <t>Homes expected to close during 2027, to the nearest 50</t>
   </si>
   <si>
-    <t>Method. Monthly closure chance for each home from a Poisson model fitted on home-months January 2016 to December 2026: year of licence, provider aged 63 or more and 68 or more, June to August, and the June to August before the provider's youngest own child starts kindergarten. Each home licensed on 31 December 2026 is carried month by month through 2027 and its chances of closing are summed.</t>
-  </si>
-  <si>
-    <t>In the record, 905 homes were open on 1 June of the summer before their youngest own child's kindergarten year and 401 of them closed by 31 August (44 per cent); in other months a home's chance of closing was well under 1 per cent a month.</t>
+    <t>Method. Monthly closure chance for each home from a Poisson model fitted on home-months January 2016 to December 2026: year of licence, provider aged 63 or more and 68 or more, June to August, and the June to August before the provider's youngest own child starts kindergarten. Each home licensed on 31 December 2026 is carried month by month through 2027 and its chances of closing are summed. Logit, straight-line and no tenure terms, fits from 2020 or 2022, rate readings and annual rates give 437 to 464; the forecast is their centre.</t>
+  </si>
+  <si>
+    <t>In the record, 903 homes were open on 1 June of the summer before their youngest own child's kindergarten year and 459 of them closed by 31 August (51 per cent); in other months a home's chance of closing was well under 1 per cent a month.</t>
   </si>
   <si>
     <t>Licensing record by year</t>
@@ -562,7 +562,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>3081</v>
+        <v>3051</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -570,7 +570,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -581,7 +581,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="60" customHeight="1">
+    <row r="9" spans="1:3" ht="78" customHeight="1">
       <c r="A9" s="6" t="s">
         <v>5</v>
       </c>
@@ -612,10 +612,10 @@
         <v>2016</v>
       </c>
       <c r="B14" s="3">
-        <v>1913</v>
+        <v>1917</v>
       </c>
       <c r="C14" s="3">
-        <v>195</v>
+        <v>212</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -623,10 +623,10 @@
         <v>2017</v>
       </c>
       <c r="B15" s="3">
-        <v>1986</v>
+        <v>1973</v>
       </c>
       <c r="C15" s="3">
-        <v>225</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -634,10 +634,10 @@
         <v>2018</v>
       </c>
       <c r="B16" s="3">
-        <v>2023</v>
+        <v>2029</v>
       </c>
       <c r="C16" s="3">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -645,10 +645,10 @@
         <v>2019</v>
       </c>
       <c r="B17" s="3">
-        <v>2060</v>
+        <v>2062</v>
       </c>
       <c r="C17" s="3">
-        <v>221</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -656,10 +656,10 @@
         <v>2020</v>
       </c>
       <c r="B18" s="3">
-        <v>2094</v>
+        <v>2079</v>
       </c>
       <c r="C18" s="3">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -667,10 +667,10 @@
         <v>2021</v>
       </c>
       <c r="B19" s="3">
-        <v>2050</v>
+        <v>2031</v>
       </c>
       <c r="C19" s="3">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -678,10 +678,10 @@
         <v>2022</v>
       </c>
       <c r="B20" s="3">
-        <v>2064</v>
+        <v>2050</v>
       </c>
       <c r="C20" s="3">
-        <v>233</v>
+        <v>249</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -689,10 +689,10 @@
         <v>2023</v>
       </c>
       <c r="B21" s="3">
-        <v>2128</v>
+        <v>2098</v>
       </c>
       <c r="C21" s="3">
-        <v>271</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -700,10 +700,10 @@
         <v>2024</v>
       </c>
       <c r="B22" s="3">
-        <v>3081</v>
+        <v>3042</v>
       </c>
       <c r="C22" s="3">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -711,10 +711,10 @@
         <v>2025</v>
       </c>
       <c r="B23" s="3">
-        <v>3127</v>
+        <v>3093</v>
       </c>
       <c r="C23" s="3">
-        <v>282</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -722,10 +722,10 @@
         <v>2026</v>
       </c>
       <c r="B24" s="3">
-        <v>3132</v>
+        <v>3080</v>
       </c>
       <c r="C24" s="3">
-        <v>322</v>
+        <v>300</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -770,7 +770,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="3">
-        <v>124773</v>
+        <v>124785</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -778,7 +778,7 @@
         <v>17</v>
       </c>
       <c r="B6" s="3">
-        <v>131302</v>
+        <v>129743</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -786,7 +786,7 @@
         <v>18</v>
       </c>
       <c r="B7" s="9">
-        <v>256075</v>
+        <v>254528</v>
       </c>
     </row>
   </sheetData>
@@ -835,16 +835,16 @@
         <v>26</v>
       </c>
       <c r="B5" s="3">
-        <v>261011</v>
+        <v>314136</v>
       </c>
       <c r="C5" s="3">
-        <v>284679</v>
+        <v>344319</v>
       </c>
       <c r="D5" s="3">
-        <v>301788</v>
+        <v>365748</v>
       </c>
       <c r="E5" s="3">
-        <v>351377</v>
+        <v>361863</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -852,16 +852,16 @@
         <v>27</v>
       </c>
       <c r="B6" s="3">
-        <v>930268</v>
+        <v>926889</v>
       </c>
       <c r="C6" s="3">
-        <v>956164</v>
+        <v>967737</v>
       </c>
       <c r="D6" s="3">
-        <v>950014</v>
+        <v>939916</v>
       </c>
       <c r="E6" s="3">
-        <v>968166</v>
+        <v>941483</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -869,16 +869,16 @@
         <v>28</v>
       </c>
       <c r="B7" s="3">
-        <v>331513</v>
+        <v>312315</v>
       </c>
       <c r="C7" s="3">
-        <v>335325</v>
+        <v>323669</v>
       </c>
       <c r="D7" s="3">
-        <v>366990</v>
+        <v>346040</v>
       </c>
       <c r="E7" s="3">
-        <v>368805</v>
+        <v>362450</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -886,16 +886,16 @@
         <v>29</v>
       </c>
       <c r="B8" s="3">
-        <v>394956</v>
+        <v>437045</v>
       </c>
       <c r="C8" s="3">
-        <v>413421</v>
+        <v>459630</v>
       </c>
       <c r="D8" s="3">
-        <v>424992</v>
+        <v>476528</v>
       </c>
       <c r="E8" s="3">
-        <v>478850</v>
+        <v>490882</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -903,16 +903,16 @@
         <v>30</v>
       </c>
       <c r="B9" s="3">
-        <v>431566</v>
+        <v>336954</v>
       </c>
       <c r="C9" s="3">
-        <v>461036</v>
+        <v>378870</v>
       </c>
       <c r="D9" s="3">
-        <v>453954</v>
+        <v>387704</v>
       </c>
       <c r="E9" s="3">
-        <v>454203</v>
+        <v>448685</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -920,16 +920,16 @@
         <v>31</v>
       </c>
       <c r="B10" s="9">
-        <v>2349314</v>
+        <v>2327339</v>
       </c>
       <c r="C10" s="9">
-        <v>2450625</v>
+        <v>2474225</v>
       </c>
       <c r="D10" s="9">
-        <v>2497738</v>
+        <v>2515936</v>
       </c>
       <c r="E10" s="9">
-        <v>2621401</v>
+        <v>2605363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task176): asks rebuilt as three tables of ten on three devices, waiting on round 5 readers and judge
Round 4 approved the call and the judge's determinism; reader G cracked the money device, which carried 20 of 22 ask
figures. The policy now pays each home the amounts of its own lines (the care_days split closed); the device-free
child-days table is dropped; money, food program meals and split care each take ten cells by region and half on
devices of different kinds. Pair 37.7, each single crack 30.3 off the call. Call and every call figure unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task176/golden/fcc_closures_2027.xlsx
+++ b/task176/golden/fcc_closures_2027.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Forecast 2027" sheetId="1" r:id="rId1"/>
-    <sheet name="Subsidy child-days" sheetId="2" r:id="rId2"/>
-    <sheet name="Subsidy payments" sheetId="3" r:id="rId3"/>
-    <sheet name="Notes" sheetId="4" r:id="rId4"/>
+    <sheet name="Subsidy payments" sheetId="2" r:id="rId2"/>
+    <sheet name="Food program meals" sheetId="3" r:id="rId3"/>
+    <sheet name="Split care" sheetId="4" r:id="rId4"/>
+    <sheet name="Notes" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="31">
   <si>
     <t>About 450 of the 3,051 licensed family child care homes are expected to close during 2027</t>
   </si>
@@ -55,16 +56,13 @@
     <t>Kindergarten year as in the CCAP provider payment policy, section 6 (a child turning five on or before 1 September starts that September). Homes are small and large family child care homes (Title 170, 6.40.010). Sources: licensing extract of 8 January 2027; capacity worksheets 2016 to 2026.</t>
   </si>
   <si>
-    <t>Child-days of subsidised care in family child care homes, Allerton, 2026</t>
-  </si>
-  <si>
-    <t>CCAP payment lines, SFCC and LFCC providers, lines not voided; each child counted once on a day (Monday to Friday) whatever the number of homes paid for that day.</t>
-  </si>
-  <si>
-    <t>Half of 2026</t>
-  </si>
-  <si>
-    <t>Child-days</t>
+    <t>Money the subsidy paid to family child care homes, 2026 payment runs (USD)</t>
+  </si>
+  <si>
+    <t>CCAP remittances for SFCC and LFCC homes by the date of the payment run and the region of the home that gave the care; voided remittances out, their reissues in; each remittance counted once (number, run and county office), each home paid the amounts of its own lines.</t>
+  </si>
+  <si>
+    <t>Region</t>
   </si>
   <si>
     <t>January to June</t>
@@ -73,30 +71,6 @@
     <t>July to December</t>
   </si>
   <si>
-    <t>2026</t>
-  </si>
-  <si>
-    <t>Money the subsidy paid to family child care homes, 2026 payment runs (USD)</t>
-  </si>
-  <si>
-    <t>CCAP remittances for SFCC and LFCC homes by the date of the payment run and the region of the home that gave the care; voided remittances out, their reissues in; each remittance counted once (number, run and county office), a remittance for homes in several regions shared by its lines' pay.</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>January to March</t>
-  </si>
-  <si>
-    <t>April to June</t>
-  </si>
-  <si>
-    <t>July to September</t>
-  </si>
-  <si>
-    <t>October to December</t>
-  </si>
-  <si>
     <t>Region 1 North</t>
   </si>
   <si>
@@ -113,6 +87,18 @@
   </si>
   <si>
     <t>Allerton</t>
+  </si>
+  <si>
+    <t>Meals and snacks claimed for family child care homes, 2026</t>
+  </si>
+  <si>
+    <t>CACFP claims for home sites by month of service; each claim (sponsor and claim number) at its latest filing; breakfasts, lunches, suppers and snacks.</t>
+  </si>
+  <si>
+    <t>Children in split care between two family child care homes, 2026</t>
+  </si>
+  <si>
+    <t>Children paid at two homes for the same days under a split authorisation (CCAP policy sections 2 and 3); a move's notice days are not split care. A child in split care in both halves is in both columns.</t>
   </si>
   <si>
     <t>Prepared 14 January 2027 from the January 2027 supply folder (licensing extract of 8 January 2027).</t>
@@ -740,53 +726,98 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="2" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:3">
       <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="C4" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3">
-        <v>124785</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>642814</v>
+      </c>
+      <c r="C5" s="3">
+        <v>690799</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3">
-        <v>129743</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="9">
-        <v>254528</v>
+        <v>1858868</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1811135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="3">
+        <v>621586</v>
+      </c>
+      <c r="C7" s="3">
+        <v>684310</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="3">
+        <v>874959</v>
+      </c>
+      <c r="C8" s="3">
+        <v>925906</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="3">
+        <v>698708</v>
+      </c>
+      <c r="C9" s="3">
+        <v>798228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="9">
+        <v>4696935</v>
+      </c>
+      <c r="C10" s="9">
+        <v>4910378</v>
       </c>
     </row>
   </sheetData>
@@ -796,140 +827,98 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="5" width="16.7109375" customWidth="1"/>
+    <col min="2" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3">
+        <v>379629</v>
+      </c>
+      <c r="C5" s="3">
+        <v>386596</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1184702</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1182405</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="B7" s="3">
+        <v>487331</v>
+      </c>
+      <c r="C7" s="3">
+        <v>490405</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="7" t="s">
+      <c r="B8" s="3">
+        <v>543358</v>
+      </c>
+      <c r="C8" s="3">
+        <v>556773</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B9" s="3">
+        <v>475902</v>
+      </c>
+      <c r="C9" s="3">
+        <v>476875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="3">
-        <v>314136</v>
-      </c>
-      <c r="C5" s="3">
-        <v>344319</v>
-      </c>
-      <c r="D5" s="3">
-        <v>365748</v>
-      </c>
-      <c r="E5" s="3">
-        <v>361863</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="3">
-        <v>926889</v>
-      </c>
-      <c r="C6" s="3">
-        <v>967737</v>
-      </c>
-      <c r="D6" s="3">
-        <v>939916</v>
-      </c>
-      <c r="E6" s="3">
-        <v>941483</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="3">
-        <v>312315</v>
-      </c>
-      <c r="C7" s="3">
-        <v>323669</v>
-      </c>
-      <c r="D7" s="3">
-        <v>346040</v>
-      </c>
-      <c r="E7" s="3">
-        <v>362450</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="3">
-        <v>437045</v>
-      </c>
-      <c r="C8" s="3">
-        <v>459630</v>
-      </c>
-      <c r="D8" s="3">
-        <v>476528</v>
-      </c>
-      <c r="E8" s="3">
-        <v>490882</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="3">
-        <v>336954</v>
-      </c>
-      <c r="C9" s="3">
-        <v>378870</v>
-      </c>
-      <c r="D9" s="3">
-        <v>387704</v>
-      </c>
-      <c r="E9" s="3">
-        <v>448685</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="8" t="s">
-        <v>31</v>
-      </c>
       <c r="B10" s="9">
-        <v>2327339</v>
+        <v>3070922</v>
       </c>
       <c r="C10" s="9">
-        <v>2474225</v>
-      </c>
-      <c r="D10" s="9">
-        <v>2515936</v>
-      </c>
-      <c r="E10" s="9">
-        <v>2605363</v>
+        <v>3093054</v>
       </c>
     </row>
   </sheetData>
@@ -938,6 +927,107 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="3" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3">
+        <v>37</v>
+      </c>
+      <c r="C6" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="3">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="3">
+        <v>21</v>
+      </c>
+      <c r="C8" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="3">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="9">
+        <v>103</v>
+      </c>
+      <c r="C10" s="9">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -947,22 +1037,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>